<commit_message>
feat(daekningsanalyse): gem analyser + dark slider track + renset data
- gem/navngiv analyser via POST /api/analyse/daekningsanalyse/saved
- liste over gemte analyser på upload-siden
- gem-knap i sidebar header med inputfelt
- slider track: mørk bg i stedet for hvid
- sample-data renset: kun frederiksberg kommune (0147), 389 adresser
- migration 169: daekningsanalyse_saved tabel med RLS

BIZZ-2001

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-bredbaand-kundedata.xlsx
+++ b/docs/sample-bredbaand-kundedata.xlsx
@@ -11,1254 +11,1176 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="390">
   <si>
     <t>Kundeadresse</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 37, 3. th, 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 4, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42B, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 55, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19A, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, 5. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 18, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, st. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 3. 304, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27A, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27A, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42B, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 1. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, st. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 6. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 8A, 4., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 12, st. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 47, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 2, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42B, 5. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 57, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, 5., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 62, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 44, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 70, kl. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 34, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98B, 5. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98B, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, st. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 62, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 18, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60A, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, st. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19A, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 25, kl. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 2. 206, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 6. 602, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41B, st. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 3. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 17, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 3. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 40, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 48, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 1. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 4. 404, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42A, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 55, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 56, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 24, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, st. 5, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 16, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 62, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98B, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 104, kl. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 3. 5, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 64, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 40, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27A, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 57, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98A, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 3. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 69, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42A, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 1. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, st. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27A, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 47, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 38, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 56, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, st. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 88, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 49, 4., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, 1. 28, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66A, 5., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 58, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 4. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 55, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 4. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19A, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 88, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 4. 402, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41B, st. 7, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 16, 2. 5, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 36, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 104, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 39, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 63, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66A, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 49, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 31, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 2. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 49, kl. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 4. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60A, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41B, 1. 11, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 36, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42A, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, kl. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 16, 1. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, st. 5, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, st. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 10A, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 88, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 25, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42A, 5. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 36, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 25, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41B, st. 8, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 80, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 88, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 6D, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19B, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 39, 4., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41A, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19A, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 15, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68A, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60C, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21B, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 47, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 2. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 3. 302, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 63, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, st. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 2. 209, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 2. 204, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 19A, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 28, kl. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 80, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 39, 2., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 6. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 45, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 39A, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 80, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 72, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 1. 5, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 25, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98A, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 5. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 44, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 71, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, st. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, kl. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 68B, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, kl. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 55, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 28A, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 6. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27A, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 34, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 34, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 37, st. 3, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 49, 2., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 36, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 26, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 40, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 100, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 3. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 39, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 16, 3. 7, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 98B, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 92, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42B, 3., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 42A, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 22A, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 56, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 38, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 62, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, kl. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 88, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 62, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 44, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 4, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 32, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 34, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, 6. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 74, 4., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 6B, 1. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 54, st. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 43, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 82, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 47, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, 5. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66, 5., 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 56, st. th, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 100, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 56, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 104, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 98A, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 4, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 2, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 10, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 17, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27B, st. 5, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41B, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, 1. 5, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 21B, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 49, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, 6. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 36, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, st. 6, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, 3. th, 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 41C, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 1. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 4. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60A, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 4. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 44, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 2. 201, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 2. 1, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 36, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 3. 301, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 35, st. th, 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 62, 1. tv, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 17, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 6. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 62, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 26, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 11, 7200 Grindsted</t>
+    <t>Frederiksberg Alle 56, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 2. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 4. 403, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 104, 2., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 23A, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 94, kl., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 27B, 4. 2, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 56, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 76, 3. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 78, 5. mf, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 34, st. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 25, kl. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66A, 2., 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 42A, st. 1, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 41, 2. 205, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 104, kl. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 6. 601, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 4. 405, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23A, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 2. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 4. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60A, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 26, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 98B, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 10A, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 104, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, 4. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 50, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, st. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 6. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 6. 602, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 63, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 71, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 28, 5., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 47, 3., 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 14, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 59, kl. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 41, 5. 502, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21B, 1., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 86, st. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, 2. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 80, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 21A, 5., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 53, 5., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 80, 4. th, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 50, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 51, 1. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 90, 3. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 66A, st., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 96, 2. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 28, st. tv, 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 28, 3., 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 60A, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 24, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41C, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42B, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 44, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 55, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6D, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 21A, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 12, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41B, st. 6, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, 4. th, 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 25, 4., 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 52, 4. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 60B, 1. 4, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 84, 2. th, 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 94, 4. tv, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 96, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6B, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19B, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 98B, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 57, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60C, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 39A, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 55, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, 4. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41B, 1. 11, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 2. 204, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 10A, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 3. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 28, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 28, kl. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 9, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, 2. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 26, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 10, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 59, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 59, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 55, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 2. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27A, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 5. 503, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68B, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19B, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 2. 203, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 3, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 49, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 14, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 1, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66A, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 50, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 70, kl. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 49, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 3. 304, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 26, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 47, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 59, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 39, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 2. 201, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 64, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 21A, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 69, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 1. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66A, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60A, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42B, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 44, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 18, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 50, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 44, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 15, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 32, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 56, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 48, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 6. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 3. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 4, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 2. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 52, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 6. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, st. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27A, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 34, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 96, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 32, st. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, st. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, 3. 6, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41B, st. 5, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60A, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6B, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 3. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 62, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 98B, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 55, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 47, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 5, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 1. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8A, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 31, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 11A, st., 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 98B, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 12, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19A, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 94, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 5. 502, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, st. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 18, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 7, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 56, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 74, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 45, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 4. 403, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 26, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, st. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 13, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 96, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 63, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 50, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 19B, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 3. 4, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 50, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 28A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27B, 3. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 39, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 4. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 28, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 6. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 17, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 62, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 62, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 39, 3., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 6, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 3. 303, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 12, st. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 62, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 22A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 36, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 96, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 11B, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27B, 4. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 59, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 34, 2. th, 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 90, 6. tv, 1820 Frederiksberg C</t>
+  </si>
+  <si>
+    <t>Frederiksberg Alle 29, kl., 1820 Frederiksberg C</t>
   </si>
   <si>
     <t>Frederiksberg Alle 102, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 4, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 16, 3. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 70, kl. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 59, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 35, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 15, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 6. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 44, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 40, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 34, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 9, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 15, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 47, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8A, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 100, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 23, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41B, 1. 10, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, 5., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 17, 1., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 5. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 4. 404, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, 3. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 10A, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 6. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 4. 407, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27B, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 68A, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 2, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 96, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, 5. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 82, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 32, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 78, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, st. 1, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 90, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42B, 2., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, kl. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 55, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 15, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 37, st. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 41, 2. 208, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 20, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42B, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8, 4., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 84, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 43, 1. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 66, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, kl., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 54, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 51, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 7, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 80, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, 4. 7, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 29, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 53, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 5, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 104, st., 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, 4. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 60B, 2. 3, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 2, 7200 Grindsted</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 25, 2. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 49, kl. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, st. 2, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 92, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 27B, 1. 5, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 72, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 88, st. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 76, 3. mf, 1820 Frederiksberg C</t>
-  </si>
-  <si>
     <t>Frederiksberg Alle 52, st. 3, 1820 Frederiksberg C</t>
   </si>
   <si>
-    <t>Frederiksberg Alle 53, 1. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 56, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 42A, 4. tv, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 34, st. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 44, 2. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 8, 6700 Esbjerg</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 86, 3. th, 1820 Frederiksberg C</t>
-  </si>
-  <si>
-    <t>Frederiksberg Alle 58, 2. tv, 1820 Frederiksberg C</t>
+    <t>Frederiksberg Alle 40, st. th, 1820 Frederiksberg C</t>
   </si>
 </sst>
 </file>
@@ -1639,7 +1561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A416"/>
+  <dimension ref="A1:A390"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
@@ -3595,136 +3517,6 @@
         <v>389</v>
       </c>
     </row>
-    <row r="391" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A391" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="392" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A392" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="393" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A393" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="394" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A394" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="395" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A395" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="396" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A396" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="397" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A397" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="398" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A398" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="399" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A399" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="400" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A400" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="401" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A401" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="402" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A402" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="403" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A403" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="404" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A404" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="405" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A405" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="406" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A406" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="407" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A407" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="408" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A408" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="409" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A409" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="410" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A410" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="411" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A411" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="412" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A412" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="413" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A413" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="414" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A414" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="415" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A415" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="416" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A416" t="s">
-        <v>415</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>